<commit_message>
Product Backlog draft modified
</commit_message>
<xml_diff>
--- a/protoflow/documentazione/process/Product_Backlog.xlsx
+++ b/protoflow/documentazione/process/Product_Backlog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dati\_Laurea Magistrale ISI\Esami\07-Paradigmi di Programmazione e Sviluppo (6)\Progetto\ProtoFlow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dati\_Laurea Magistrale ISI\Esami\07-Paradigmi di Programmazione e Sviluppo (6)\PPS-25-ProtoFlow\protoflow\documentazione\process\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17D84D4-15C8-4F7D-BB51-C429C62DBF7E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D45F580-9F38-46AF-88EF-6A631ACB1324}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12312" windowHeight="6096" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -450,14 +450,14 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -747,7 +747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.109375" style="3" customWidth="1"/>
@@ -759,13 +759,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
@@ -849,7 +849,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="67.8" customHeight="1" x14ac:dyDescent="0.25">
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -883,7 +883,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -917,14 +917,14 @@
         <v>0</v>
       </c>
       <c r="E12" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="16" t="s">
         <v>80</v>
       </c>
       <c r="C13" s="12" t="s">
@@ -934,7 +934,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>